<commit_message>
chore: add agent revenue ops task system
</commit_message>
<xml_diff>
--- a/ops/agent-native-revenue/battlelabs-agent-product-dashboard.xlsx
+++ b/ops/agent-native-revenue/battlelabs-agent-product-dashboard.xlsx
@@ -9,6 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Metrics" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Queue" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Linear Import" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keyword Map" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -61,12 +64,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -602,7 +606,6 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -615,7 +618,6 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -628,7 +630,6 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -641,7 +642,6 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -654,7 +654,6 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -667,7 +666,1747 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="43" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Task ID</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Queue</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Owner Agent</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Dependency</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Target Artifact</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BL-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Launch Kit Baseline</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Freeze Memory Journal Gift Launch Kit SKU</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Controller Agent</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>SKU, buyer, promise, price ladder, deliverables, and compliance notes are documented</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>src/lib/memory-journal-product.ts</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>First agent-native SKU exists</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BL-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Launch Kit Baseline</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Verify generated product assets</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>QA Agent</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>BL-001</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Free sample PDF, full PDF, preview PDF, CSVs, listing copy, and promo SVGs exist and open</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>public/products/memory-journal-gift-kit</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Verified by tests/build and PDF page-count check</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BL-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Launch Kit Baseline</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Create launch pack</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Distribution Agent</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>BL-001</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>SEO copy, warm email, post variants, refund terms, and checkout setup instructions exist</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>ops/agent-native-revenue/memory-journal-launch-pack.md</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Ready for marketplace setup</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BL-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Drive Operations</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Import product dashboard to Google Sheets</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Orchestrator Agent</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>BL-002</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Dashboard workbook is uploaded or manually imported to Google Sheets with tabs preserved</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>ops/agent-native-revenue/battlelabs-agent-product-dashboard.xlsx</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Drive connector returned 403; use browser/manual import until OAuth scope is fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BL-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Checkout</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Create $9 intro checkout link</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Payment Agent</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>BL-003</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PayPal, Payhip, or Gumroad link exists and is added to NEXT_PUBLIC_MEMORY_JOURNAL_CHECKOUT_URL</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>.env.local</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>No paid subscription or ad spend allowed</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BL-006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Publish</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Publish landing page with checkout link</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Build Agent</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>BL-005</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>/memory-journal-gift-kit displays checkout CTA and assets remain downloadable</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>src/app/memory-journal-gift-kit/page.tsx</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Current page works; checkout env var is pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BL-007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SEO Foundation</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Create keyword map</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Opportunity Agent</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>BL-003</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>30-50 keywords include intent, platform, title usage, and priority</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>ops/agent-native-revenue/seo-keyword-map.csv</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Use memory-journal gift and KDP creator intent</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BL-008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Marketplace Setup</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Prepare marketplace listing fields</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Marketplace Agent</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>BL-007</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>KDP, Payhip/Gumroad, and Pinterest destination copy can be pasted with no missing fields</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>ops/agent-native-revenue/marketplace-listings.md</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>No bestseller/review/income claims</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BL-009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Organic Distribution</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Create Pinterest and social post queue</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Design Agent</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>BL-007</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>25 pin concepts, 8 board names, 10 captions, 5 short scripts, and CTA rules exist</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>ops/agent-native-revenue/distribution-task-list.md</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>No spam or paid promotion</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>BL-010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Warm Outreach</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Create warm-only Gmail draft set</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Gmail Agent</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>BL-003</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>5 templates exist with real relationship reason, one ask, opt-out language, and no attachments by default</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>ops/agent-native-revenue/warm-gmail-drafts.md</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Do not send without recipient-specific context</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BL-011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Community Distribution</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Find organic placement opportunities</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Community Agent</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>BL-008</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>30 opportunities include URL, audience, rules, allowed promo format, contact method, pitch, and risk level</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>ops/agent-native-revenue/community-opportunities.csv</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Ask mods when unsure</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BL-012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Measurement</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Track launch metrics</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Metrics Agent</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>BL-006</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Views, downloads, checkout clicks, sales, refunds, net revenue, and decisions are updated</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>ops/agent-native-revenue/battlelabs-agent-product-dashboard.xlsx</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Use Google Sheet when import is available</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>BL-013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Kill improve or clone SKU</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Controller Agent</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>BL-012</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Decision uses opt-ins, checkout clicks, sales, refunds, buyer language, and build hours</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>ops/agent-native-revenue/decision-log.md</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Clone only from evidence</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="43" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Issue ID</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Labels</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BL-004</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Import product dashboard to Google Sheets</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Upload or manually import ops/agent-native-revenue/battlelabs-agent-product-dashboard.xlsx into Google Sheets. Preserve Product Metrics and QA Checklist tabs. Current blocker: Drive connector returned 403, so use browser/manual import or reconnect Drive scope.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>drive,sheets,ops,blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BL-005</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Create intro checkout link</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Create a $9 intro product link for Memory Journal Gift Launch Kit through PayPal, Payhip, or Gumroad. Add the link to NEXT_PUBLIC_MEMORY_JOURNAL_CHECKOUT_URL and verify tracked checkout URL works.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>checkout,revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BL-006</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Publish landing page with checkout link</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Deploy /memory-journal-gift-kit after checkout link is configured. Acceptance: page loads, free sample downloads, full paid assets are ready for delivery, and checkout CTA points to the live product.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>publish,web,revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BL-007</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Create SEO keyword map</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Create 30-50 keywords for memory journal gift intent. Include keyword, intent, platform, title usage, priority, and notes. Avoid keyword stuffing.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>seo,research</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BL-008</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Prepare marketplace listing fields</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Create paste-ready listing fields for Payhip or Gumroad, KDP later, and Pinterest destination copy. Include title, subtitle, description, price, image captions, refund/usage copy, and compliance notes.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>marketplace,copy</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BL-009</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Create Pinterest and social post queue</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Produce 25 pin concepts, 8 board names, 10 captions, 5 short video scripts, 5 carousel outlines, and CTA rules. Use product/sample-page visuals and no fake scarcity.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>distribution,design</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BL-010</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Create warm-only Gmail draft set</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Draft 5 warm email templates: feedback request, soft launch, gift-guide pitch, creator collaboration, and follow-up. Each must require a real relationship reason and easy opt-out language.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>gmail,outreach</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BL-011</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Find organic placement opportunities</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Research 30 rule-compliant communities/blogs/newsletters/group boards. Track URL, audience, rules, contact method, suggested pitch, and risk level.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>community,distribution</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BL-012</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Track launch metrics</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Update the dashboard with views, sample downloads, checkout clicks, sales, refunds, net revenue, conversion rate, and next action. Use local workbook until Google Sheets import works.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>metrics,revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>BL-013</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Decide kill improve or clone</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Use evidence to decide whether to improve the current SKU, clone another recipient variant, or switch lanes. Clone only when sales, checkout clicks, opt-ins, or buyer language justify it.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>controller,decision</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="43" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="41" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Keyword</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Intent</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Title Usage</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>memory journal gift</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>KDP Payhip Pinterest</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Primary product headline</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Narrow gift intent</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>grandma memory journal</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Gift buyer KDP seller</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>KDP Payhip Pinterest</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>SKU title and pin title</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>First recipient angle</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>guided memory journal</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>KDP Blog Pinterest</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Subtitle or FAQ</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Explains format</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>family keepsake journal</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>KDP Pinterest</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Alternative title</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Emotional positioning</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>questions to ask your grandmother journal</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Gift buyer Pinterest</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Pinterest pin and FAQ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Long-tail prompt intent</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>grandparent memory book</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>KDP Pinterest</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Variant title</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Adjacent variant</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>memory book for mom</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>KDP Pinterest</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Variant research</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Potential clone</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>family stories keepsake book</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>KDP Blog</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>SEO paragraph</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Preservation angle</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>legacy journal for parents</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>KDP Blog</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Variant research</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Use carefully around grief/sentiment</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>printable memory journal interior</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Creator</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>KDP Payhip Blog</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Creator-facing product copy</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Matches digital-product buyer</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>KDP memory journal template</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Creator</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>KDP Payhip Blog</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Creator-facing title</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Buyer intent for kit</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>guided journal prompts for grandparents</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Gift buyer Pinterest</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Pin title and sample CTA</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Content-led traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>family history journal prompts</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Creator gift buyer</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Blog Pinterest</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Value post title</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Useful non-promotional content</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>meaningful gift for grandma</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Pinterest Blog</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Gift-guide pin</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Soft consumer angle</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Mother's Day memory journal</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Seasonal gift buyer</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Pinterest Blog</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Seasonal pin</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Use near holiday windows</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Christmas gift memory journal</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Seasonal gift buyer</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Pinterest Blog</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Seasonal pin</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Use near holiday windows</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>retirement memory journal</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Pinterest Blog</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Variant research</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Occasion niche</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>bereavement memory journal</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Pinterest Blog</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Variant research</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Sensitive wording; avoid therapy claims</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>family reunion keepsake journal</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Pinterest Blog</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Value post</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Occasion angle</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>gift for aging parents</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Pinterest Blog</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Gift-guide angle</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Use respectfully</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: ship no-spend metrics + delivery flow
</commit_message>
<xml_diff>
--- a/ops/agent-native-revenue/battlelabs-agent-product-dashboard.xlsx
+++ b/ops/agent-native-revenue/battlelabs-agent-product-dashboard.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -456,106 +456,172 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Page URL</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Views</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Sample Downloads</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Free Sample Clicks</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Checkout Clicks</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Refunds</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Gross Revenue</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Net Revenue</t>
-        </is>
-      </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Build Hours</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Revenue Per Build Hour</t>
-        </is>
-      </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Conversion Rate</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
           <t>Next Action</t>
         </is>
       </c>
+      <c r="L1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>KDP-SCORECARD-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>KDP Niche Scorecard Generator + KDP Launch Report</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>/kdp-niche-scorecard</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>The $19 PayPal Hosted Button is wired (XBV9JNJS6SPJE). Buyer-ready package exists at deliverables/kdp-launch-report-kit.zip and Drive delivery link is uploaded + direct-download verified; see ops/agent-native-revenue/kdp-report-delivery-handoff.md. Metrics are logged via /api/metrics/event (page_view, free_sample_click, checkout_click); see ops/agent-native-revenue/metrics-playbook.md. Next: on 2026-04-28 03:01 ET capture the live Product Hunt URL, monitor comments, then pull logs and count metrics deterministically with scripts/summarize-metric-events.ps1; update ops/agent-native-revenue/placement-tracking-log.csv + this dashboard after +24h.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BL-001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>Memory Journal Gift Launch Kit</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2">
-        <f>IF(I2&gt;0,H2/I2,0)</f>
-        <v/>
-      </c>
-      <c r="K2">
-        <f>IF(B2&gt;0,E2/B2,0)</f>
-        <v/>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Launch</t>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>/memory-journal-gift-kit</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Checkout is live at /memory-journal-gift-kit/checkout via PayPal Buttons. Metrics are logged via /api/metrics/event (page_view, free_sample_click, checkout_click); see ops/agent-native-revenue/metrics-playbook.md. Next: pick one low-risk no-spend distribution push, capture 24h metrics in ops/agent-native-revenue/metrics-snapshot-log.csv, then decide whether to improve the page or expand distribution.</t>
         </is>
       </c>
     </row>
@@ -606,6 +672,7 @@
           <t>Open</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -618,6 +685,7 @@
           <t>Open</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -630,6 +698,7 @@
           <t>Open</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -642,6 +711,7 @@
           <t>Open</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -654,6 +724,7 @@
           <t>Open</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -666,6 +737,7 @@
           <t>Open</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -678,7 +750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -923,7 +995,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Drive connector returned 403; use browser/manual import until OAuth scope is fixed</t>
+          <t>Drive connector returned 403 (including Google Drive _import_spreadsheet on 2026-04-26). Use browser/manual import. No-connector fallback: import ops/agent-native-revenue/dashboard-tabs-import-pack-2026-04-26.zip as tabs (see dashboard-tabs/IMPORT_MANIFEST.md).</t>
         </is>
       </c>
     </row>
@@ -955,22 +1027,22 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>PayPal, Payhip, or Gumroad link exists and is added to NEXT_PUBLIC_MEMORY_JOURNAL_CHECKOUT_URL</t>
+          <t>Internal checkout route exists at /memory-journal-gift-kit/checkout with PayPal capture for $9 and the landing CTA routes into it by default</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Accepted</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>.env.local</t>
+          <t>src/app/memory-journal-gift-kit/checkout/page.tsx</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>No paid subscription or ad spend allowed</t>
+          <t>Shipped internal PayPal checkout route so we are not blocked on external Payhip/Gumroad credentials. Optional: override NEXT_PUBLIC_MEMORY_JOURNAL_CHECKOUT_URL with a delivery provider link later.</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1079,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Accepted</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1017,7 +1089,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Current page works; checkout env var is pending</t>
+          <t>Landing page now defaults checkout CTA to /memory-journal-gift-kit/checkout. Checkout page captures payment via PayPal Buttons and shows the download links.</t>
         </is>
       </c>
     </row>
@@ -1054,7 +1126,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Accepted</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1064,7 +1136,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Use memory-journal gift and KDP creator intent</t>
+          <t>Expanded to 50 keywords on 2026-04-26</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1173,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Accepted</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1111,7 +1183,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>No bestseller/review/income claims</t>
+          <t>Paste-ready fields plus tags added 2026-04-26</t>
         </is>
       </c>
     </row>
@@ -1148,17 +1220,17 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>ops/agent-native-revenue/distribution-task-list.md</t>
+          <t>ops/agent-native-revenue/pinterest-social-post-queue-memory-journal.md</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>No spam or paid promotion</t>
+          <t>Delivered post queue + CTA rules. No spam or paid promotion.</t>
         </is>
       </c>
     </row>
@@ -1195,7 +1267,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1205,7 +1277,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Do not send without recipient-specific context</t>
+          <t>2026-04-26 ET: 5 warm-only drafts shipped; each requires a real relationship reason; no attachments by default. Do not send without recipient-specific context.</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1314,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1252,7 +1324,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Ask mods when unsure</t>
+          <t>Completed 2026-04-26 ET. Ask mods when unsure.</t>
         </is>
       </c>
     </row>
@@ -1289,17 +1361,17 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>ops/agent-native-revenue/battlelabs-agent-product-dashboard.xlsx</t>
+          <t>ops/agent-native-revenue/battlelabs-agent-product-dashboard.csv</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Use Google Sheet when import is available</t>
+          <t>No-spend measurement pipeline shipped: POST /api/metrics/event logs page_view/free_sample_click/checkout_click events for KDP + Memory Journal pages (see ops/agent-native-revenue/metrics-playbook.md). Baseline snapshot exists in ops/agent-native-revenue/metrics-snapshot-log.csv. Next: after placements/distribution pushes, update +24h snapshots (KDP-SCORECARD-008 and new Memory Journal snapshot entries).</t>
         </is>
       </c>
     </row>
@@ -1347,6 +1419,523 @@
       <c r="I14" t="inlineStr">
         <is>
           <t>Clone only from evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>KDP-SCORECARD-001</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>KDP Niche Scorecard</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Define launch plan</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Controller Agent</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Buyer, promise, price, compliance, and kill rules are documented</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>ops/agent-native-revenue/kdp-scorecard-launch-plan.md</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Completed by agent sprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>KDP-SCORECARD-002</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>KDP Niche Scorecard</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Build deterministic score logic</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Build Agent</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>KDP-SCORECARD-001</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Reusable score model exists with thresholds and test coverage</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>src/lib/kdp-scorecard.ts</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Tested with Vitest</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>KDP-SCORECARD-003</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>KDP Niche Scorecard</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Publish free scorecard page</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Build Agent</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>KDP-SCORECARD-002</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Free tool page exists with paid report CTA and no-guarantee disclaimer</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>src/app/kdp-niche-scorecard/page.tsx</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Built and browser-smoke-tested locally. 2026-04-26: $19 KDP Launch Report PayPal Hosted Button XBV9JNJS6SPJE wired into the paid CTA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>KDP-SCORECARD-004</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>KDP Niche Scorecard</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Create free and paid report sources</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Build Agent</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>KDP-SCORECARD-003</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Free sample, public preview, and buyer-ready paid ZIP package exist</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>deliverables/kdp-launch-report-kit.zip</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-04-26: Repackaged paid deliverable outside public directory with PDF, Markdown report, CSVs, listing starter, checklist, and license/refund/disclosure notes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>KDP-SCORECARD-010</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>KDP Niche Scorecard</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Verify Drive delivery link</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Delivery Agent</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>KDP-SCORECARD-004</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Paid ZIP is uploaded to Drive with anyone-with-link reader permission and unauthenticated download test passes</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>ops/agent-native-revenue/kdp-report-delivery-handoff.md</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-04-26: Uploaded KDP Launch Report Kit ZIP to Drive, set anyoneWithLink reader, direct-download size matched local ZIP, and ZIP entries were verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>KDP-SCORECARD-011</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>KDP Niche Scorecard</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Verify PayPal payment-to-download flow</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Payment Agent</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>KDP-SCORECARD-010</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>A buyer can complete checkout and see or receive the Drive delivery link without manual intervention</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>PayPal Hosted Button XBV9JNJS6SPJE</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Blocked until PayPal post-payment delivery/return instructions are configured and a real checkout test is run by a human operator. Agents do not spend money per eval gates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>KDP-SCORECARD-005</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>KDP Niche Scorecard</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Prepare organic distribution</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Distribution Agent</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>KDP-SCORECARD-003</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>SEO and social launch tasks are added for the new SKU</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>ops/agent-native-revenue/distribution-task-list.md</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Verified 2026-04-26 ET: distribution tasks + drafts exist (see distribution-task-list.md + first-three-organic-placement-packet.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>KDP-SCORECARD-006</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>KDP Niche Scorecard</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Run eval-gated self-improvement loop</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Controller Agent</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>KDP-SCORECARD-005</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Product evals pass before changes are promoted</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>ops/agent-native-revenue/self-improvement-eval-gates.md</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-04-26 08:00 ET: Shipped interactive scorecard sliders + shareable link on /kdp-niche-scorecard and repaired eval distribution gate check. Gates: npm test/lint/build/eval:products PASS. 2026-04-26 10:00 ET: Updated scorecard checklist link wording and aligned Product Hunt tracking artifacts to use canonical https://battlelabs.live/kdp-niche-scorecard. Gates: npm test/lint/build/eval:products PASS. 2026-04-26 11:11 ET: Added /kdp-niche-scorecard/checklist (public-friendly) and redirected /kdp-niche-scorecard/rubric; updated launch artifacts to reference the checklist URL. Gates: npm test/lint/build/eval:products PASS. 2026-04-26 12:04 ET: Added copy/paste post-text template to the interactive widget share section and shipped ops/agent-native-revenue/kdp-scorecard-clean-share-examples.md. Gates: npm test/lint/build/eval:products PASS. 2026-04-26 14:05 ET: Added dedicated Open Graph + Twitter images for /kdp-niche-scorecard/checklist to improve link previews ahead of Product Hunt. Gates: npm test/lint/build/eval:products PASS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>KDP-SCORECARD-007</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>KDP Niche Scorecard</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Publish first 3 placements</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Distribution Agent</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>KDP-SCORECARD-005</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Product Hunt, Show HN, and r/SideProject posts are published (or recorded as blocked/filtered by platform access or policy gates) with placement URLs + timestamps</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>ops/agent-native-revenue/first-three-organic-placement-packet.md</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-04-26 ET: Product Hunt scheduled for 2026-04-28 03:01 ET (capture final PH URL once live). HN authenticated submit hit /showlim and should not be retried. Reddit r/SideProject submitted then removed by Reddit filters at https://www.reddit.com/r/SideProject/comments/1sw788w/i_built_a_free_kdp_niche_scorecard_and_want/. Next: monitor Product Hunt launch and continue lower-risk no-spend placements; do not evade Reddit/HN filters.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>KDP-SCORECARD-008</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>KDP Niche Scorecard</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Update metrics after placements</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Metrics Agent</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>KDP-SCORECARD-007</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Dashboard updated with Views, Free Sample Clicks, Checkout Clicks, and next action after 24h</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>ops/agent-native-revenue/placement-tracking-log.csv</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>After 24h, update counts + any buyer language from comments. Use scripts/summarize-metric-events.ps1 to count [METRIC_EVENT] lines deterministically. If zeros, revise distribution angle before expanding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>KDP-SCORECARD-009</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>KDP Niche Scorecard</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Prepare Product Hunt listing fields</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Distribution Agent</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>KDP-SCORECARD-005</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Paste-ready Product Hunt listing fields exist and avoid internal terms like rubric</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>ops/agent-native-revenue/producthunt-listing-fields-kdp-scorecard.md</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2026-04-26 ET: Added paste-ready listing fields + maker comment + verification checklist.</t>
         </is>
       </c>
     </row>
@@ -1417,7 +2006,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Upload or manually import ops/agent-native-revenue/battlelabs-agent-product-dashboard.xlsx into Google Sheets. Preserve Product Metrics and QA Checklist tabs. Current blocker: Drive connector returned 403, so use browser/manual import or reconnect Drive scope.</t>
+          <t>Upload or manually import ops/agent-native-revenue/battlelabs-agent-product-dashboard.xlsx into Google Sheets. Preserve Product Metrics and QA Checklist tabs. No-connector fallback: import ops/agent-native-revenue/dashboard-tabs/*.csv as tabs. Current blocker: Drive connector returned 403, so use browser/manual import or reconnect Drive scope.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1449,12 +2038,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Create a $9 intro product link for Memory Journal Gift Launch Kit through PayPal, Payhip, or Gumroad. Add the link to NEXT_PUBLIC_MEMORY_JOURNAL_CHECKOUT_URL and verify tracked checkout URL works.</t>
+          <t>Create a $9 intro product link for Memory Journal Gift Launch Kit through PayPal, Payhip, or Gumroad. Add the link to NEXT_PUBLIC_MEMORY_JOURNAL_CHECKOUT_URL and verify tracked checkout URL works. Blocked on payment account credentials. Handoff: ops/agent-native-revenue/checkout-handoff-memory-journal.md</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1486,7 +2075,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1518,7 +2107,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1550,7 +2139,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1582,7 +2171,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1614,7 +2203,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1646,7 +2235,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1735,7 +2324,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
@@ -2283,7 +2872,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>retirement memory journal</t>
+          <t>gift for aging parents</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2298,24 +2887,24 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Variant research</t>
+          <t>Gift-guide angle</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Occasion niche</t>
+          <t>Use respectfully</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>bereavement memory journal</t>
+          <t>grandma memory journal gift</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2325,29 +2914,29 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Pinterest Blog</t>
+          <t>Pinterest KDP</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Variant research</t>
+          <t>Pin title and marketplace title variant</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Sensitive wording; avoid therapy claims</t>
+          <t>Direct gift phrasing</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>family reunion keepsake journal</t>
+          <t>grandmother memory journal</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2357,29 +2946,29 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Pinterest Blog</t>
+          <t>KDP Pinterest</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Value post</t>
+          <t>Title variant and backend keyword</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Occasion angle</t>
+          <t>Synonym coverage</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>gift for aging parents</t>
+          <t>grandma keepsake journal</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2389,22 +2978,982 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
+          <t>Pinterest KDP</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Pin title and backend keyword</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Giftable keepsake angle</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>grandma story journal</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Pinterest KDP</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Title variant</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Story preservation framing</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>grandma life story journal</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Pinterest KDP</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Title variant</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Life story positioning</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>grandmother interview journal</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Pinterest KDP</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Pin hook and FAQ</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Interview prompt intent</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>questions to ask grandma</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
           <t>Pinterest Blog</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Gift-guide angle</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Pin title and value post title</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Shorter query for pins</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>questions for grandma journal</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Pinterest KDP</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Pin title</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Use respectfully</t>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Journalized long-tail</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>grandma journal prompts</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Pinterest Blog</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Value post H2</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Content keyword</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>family memory journal</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>KDP Pinterest</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Title variant</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Broader family angle</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>family memories journal prompts</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Blog Pinterest</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Value post title</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Content-led traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>family story journal prompts</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Blog Pinterest</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Value post title</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Prompt intent</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>family interview questions journal</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Blog Pinterest</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Value post title</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Interview format</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>questions to ask your parents journal</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Blog Pinterest</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Variant research</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Adjacent recipient</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>memory journal for mom</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>KDP Pinterest</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Variant title research</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Clone candidate</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>grandpa memory journal</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>KDP Pinterest</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Variant title research</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Clone candidate</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>grandparent interview questions</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Blog Pinterest</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Value post title</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Non-journal phrasing</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>family history interview questions</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Blog Pinterest</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Value post title</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Evergreen content</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>keepsake journal for grandparents</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>KDP Pinterest</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Title variant</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Recipient framing</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>keepsake journal for grandma</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>KDP Pinterest</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Title variant</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Recipient framing</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>guided journal for grandma</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Gift buyer</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>KDP Pinterest</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Title variant</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Format plus recipient</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>printable memory journal PDF</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Creator</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>KDP Payhip Gumroad</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Marketplace keywords and tags</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Digital format cue</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>printable guided journal template</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Creator</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Payhip Gumroad Blog</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Creator-facing title</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Template intent</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>guided journal interior template</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Creator</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Payhip Gumroad</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Bullet section header</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Interior focus</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>KDP guided journal interior</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Creator</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>KDP Blog</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Creator-facing SEO paragraph</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>KDP-specific</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>KDP journal interior PDF</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Creator</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>KDP Blog</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Creator-facing SEO paragraph</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Format plus KDP</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>printable journal launch kit</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Creator</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Gumroad Payhip</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Benefit bullet header</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Direct kit intent</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>giftable journal niche idea</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Creator</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>SEO paragraph</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Idea validation tie-in</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>KDP gift journal niche</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Creator</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>SEO paragraph</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Positioning for creators</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>memory journal niche research</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Creator</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>SEO paragraph</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Creator research angle</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>printable keepsake journal template</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Creator</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Payhip Gumroad</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Marketplace keyword</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Keepsake plus template</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>guided keepsake journal template</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Creator</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Payhip Gumroad</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Marketplace keyword</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Template variant</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>family keepsake journal template</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Creator</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Payhip Gumroad</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Marketplace keyword</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Template variant</t>
         </is>
       </c>
     </row>

</xml_diff>